<commit_message>
chore(data-release): publish site data 2026-10-08 02:17:12 UTC
</commit_message>
<xml_diff>
--- a/diseases/d008/2026-2029.xlsx
+++ b/diseases/d008/2026-2029.xlsx
@@ -66875,13 +66875,13 @@
         </is>
       </c>
       <c r="N350" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O350" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R350" t="n">
-        <v>0.03294548870446478</v>
+        <v>0.03488345862825683</v>
       </c>
       <c r="S350" t="inlineStr">
         <is>
@@ -67020,13 +67020,13 @@
         </is>
       </c>
       <c r="N351" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O351" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R351" t="n">
-        <v>0.001937969923792046</v>
+        <v>0.003875939847584092</v>
       </c>
       <c r="S351" t="inlineStr">
         <is>
@@ -67276,7 +67276,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1377849</v>
+        <v>1377851</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-15 17:23:15 UTC
</commit_message>
<xml_diff>
--- a/diseases/d008/2026-2029.xlsx
+++ b/diseases/d008/2026-2029.xlsx
@@ -16225,13 +16225,13 @@
         </is>
       </c>
       <c r="N84" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O84" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="R84" t="n">
-        <v>0.2803464128485004</v>
+        <v>0.271001532420217</v>
       </c>
       <c r="S84" t="inlineStr">
         <is>
@@ -16384,10 +16384,10 @@
         </is>
       </c>
       <c r="N85" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O85" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="U85" t="inlineStr">
         <is>
@@ -24012,13 +24012,13 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O125" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="R125" t="n">
-        <v>0.3831400975596171</v>
+        <v>0.3737952171313338</v>
       </c>
       <c r="S125" t="inlineStr">
         <is>
@@ -24171,10 +24171,10 @@
         </is>
       </c>
       <c r="N126" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O126" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="U126" t="inlineStr">
         <is>
@@ -31550,13 +31550,13 @@
         </is>
       </c>
       <c r="N165" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O165" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="R165" t="n">
-        <v>0.3924849779879006</v>
+        <v>0.3737952171313338</v>
       </c>
       <c r="S165" t="inlineStr">
         <is>
@@ -31709,10 +31709,10 @@
         </is>
       </c>
       <c r="N166" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O166" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="U166" t="inlineStr">
         <is>
@@ -39716,13 +39716,13 @@
         </is>
       </c>
       <c r="N208" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O208" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="R208" t="n">
-        <v>0.3924849779879006</v>
+        <v>0.3737952171313338</v>
       </c>
       <c r="S208" t="inlineStr">
         <is>
@@ -39875,10 +39875,10 @@
         </is>
       </c>
       <c r="N209" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O209" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="U209" t="inlineStr">
         <is>
@@ -47488,13 +47488,13 @@
         </is>
       </c>
       <c r="N249" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="O249" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="R249" t="n">
-        <v>0.2336220107070837</v>
+        <v>0.2055873694222336</v>
       </c>
       <c r="S249" t="inlineStr">
         <is>
@@ -47647,10 +47647,10 @@
         </is>
       </c>
       <c r="N250" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="O250" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="U250" t="inlineStr">
         <is>
@@ -67934,7 +67934,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1377992</v>
+        <v>1377983</v>
       </c>
     </row>
     <row r="16">

</xml_diff>